<commit_message>
Correct retail authority evidence and render proofs
</commit_message>
<xml_diff>
--- a/research/retail-price-accuracy/mutations/dc-price-weight-duplicate-scan-v1/documents/jurisdiction-authority-map-v2.xlsx
+++ b/research/retail-price-accuracy/mutations/dc-price-weight-duplicate-scan-v1/documents/jurisdiction-authority-map-v2.xlsx
@@ -458,7 +458,7 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="27" customWidth="1" min="9" max="9"/>
@@ -2672,22 +2672,22 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Or. Rev. Stat. §§ 616.850–616.890</t>
+          <t>OAR 603-027-0180; Or. Rev. Stat. §§ 616.850–616.890</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Unit and total retail price disclosure for covered grocery commodities.</t>
+          <t>UPC/PLU scanner price-verification examinations and complementary unit-price disclosure.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.oregonlegislature.gov/bills_laws/ors/ors616.html</t>
+          <t>https://secure.sos.state.or.us/oard/view.action?ruleNumber=603-027-0180</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>official_state_statute</t>
+          <t>official_state_regulation_and_statute</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2967,22 +2967,22 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Tenn. Code Ann. § 47-26-907</t>
+          <t>Tenn. Code Ann. § 47-26-913</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>State inspection program verifies UPC charges against advertisements, labels, and shelf prices.</t>
+          <t>Prohibits misleading price representations for commodities or services sold by weight, measure, or count.</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.tn.gov/agriculture/consumers/standards.html</t>
+          <t>https://capitol.tn.gov/Archives/Joint/committees/gov-opps/RulesPackets/Rule%20Review%20Packet%20-%20July%202026.pdf</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>official_state_program</t>
+          <t>official_state_rule_packet_plus_secondary_code_text</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -3262,17 +3262,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Wash. Rev. Code § 19.94.230</t>
+          <t>Wash. Rev. Code § 19.94.390</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Prohibits misleading price representations for commodities sold by weight, measure, or count.</t>
+          <t>Prohibits misleading price representations, adopts scanner price-verification procedures, and requires consumer-visible scanner screens.</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://app.leg.wa.gov/RCW/default.aspx?cite=19.94.230</t>
+          <t>https://app.leg.wa.gov/RCW/default.aspx?cite=19.94.390</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>

</xml_diff>